<commit_message>
Sync YouTube企画案 with Drive state and add ID 39-40 (Part 3 unknown-topic ideas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RtfXaXCCtZF9HxDQKAMx27
</commit_message>
<xml_diff>
--- a/planning/YouTube企画案.xlsx
+++ b/planning/YouTube企画案.xlsx
@@ -4820,42 +4820,42 @@
       </c>
       <c r="B44" s="85" t="inlineStr">
         <is>
-          <t>実験</t>
+          <t>本命</t>
         </is>
       </c>
       <c r="C44" s="86" t="inlineStr">
         <is>
-          <t>Shorts：スピーキング8.0の私がPart 2でやらないこと3選</t>
+          <t>IELTSスピーキングPart 3の「知らない話題」は、実は7.0へのチャンスだった</t>
         </is>
       </c>
       <c r="D44" s="86" t="inlineStr">
         <is>
-          <t>IELTS Speaking（Shorts）</t>
+          <t>IELTS Speaking</t>
         </is>
       </c>
       <c r="E44" s="85" t="inlineStr">
         <is>
-          <t>実験枠</t>
+          <t>通過</t>
         </is>
       </c>
       <c r="F44" s="86" t="inlineStr">
         <is>
-          <t>Shorts上位が「スピーキング8.0の私が〜3選」型：4,012回（Shorts平均1,572の約2.6倍）、2,593回（約1.6倍）、2,123回（約1.4倍）。同じ型の続編</t>
+          <t>自チャンネル「IELTSスピーキング本番で沈黙を防ぐ練習法」1,235回＝約3.7倍、Shorts「質問の意味が一瞬分からなかった時の対処法3選」1,910回＝約1.2倍。一方「Part 3で『黙ってしまう』最大の原因とは？」は195回 → 原因論より『ピンチがチャンスに変わる』逆転の見せ方と具体策で。ID 15（答えに詰まった瞬間のリカバリー）と内容が近い</t>
         </is>
       </c>
       <c r="G44" s="86" t="inlineStr">
         <is>
-          <t>チュートリアル（Shorts）</t>
+          <t>チュートリアル×解説</t>
         </is>
       </c>
       <c r="H44" s="86" t="inlineStr">
         <is>
-          <t>明確なリスト（数字）× 親近感</t>
+          <t>トピック＋ひねり × 変身・変化</t>
         </is>
       </c>
       <c r="I44" s="86" t="inlineStr">
         <is>
-          <t>「IELTSスピーキング8.0の私が、Part 2で絶対にやらないこと3選」</t>
+          <t>「Part 3の『知らない話題』は、実は7.0へのチャンスだった」／固まった顔 → 7.0のスコア</t>
         </is>
       </c>
       <c r="J44" s="85" t="n"/>
@@ -4889,42 +4889,42 @@
       </c>
       <c r="B45" s="85" t="inlineStr">
         <is>
-          <t>実験</t>
+          <t>本命</t>
         </is>
       </c>
       <c r="C45" s="86" t="inlineStr">
         <is>
-          <t>Shorts：スピーキング8.0の私がPart 3で詰まった時に言うこと</t>
+          <t>IELTSスピーキングで知らない話題に詰まるのは英語力のせいじゃない</t>
         </is>
       </c>
       <c r="D45" s="86" t="inlineStr">
         <is>
-          <t>IELTS Speaking（Shorts）</t>
+          <t>IELTS Speaking</t>
         </is>
       </c>
       <c r="E45" s="85" t="inlineStr">
         <is>
-          <t>実験枠</t>
+          <t>通過</t>
         </is>
       </c>
       <c r="F45" s="86" t="inlineStr">
         <is>
-          <t>「IELTSスピーキング質問の意味が一瞬分からなかった時の対処法3選」1,910回（約1.2倍）＋8.0の私型の横展開</t>
+          <t>沈黙・詰まり系は自チャンネルで実績あり（沈黙を防ぐ練習法 1,235回＝約3.7倍）。ただし「〜のせいじゃない」「〜が原因じゃない」型の過去動画は控えめ：「スピーキングで詰まるのは語彙不足が原因じゃない」377回＝約1.1倍、「ライティングが伸びないのは英語力のせいじゃない」353回＝約1.1倍。ID 39と同じテーマなので、どちらかをタイトル案として統合も可</t>
         </is>
       </c>
       <c r="G45" s="86" t="inlineStr">
         <is>
-          <t>チュートリアル（Shorts）</t>
+          <t>解説×チュートリアル</t>
         </is>
       </c>
       <c r="H45" s="86" t="inlineStr">
         <is>
-          <t>明確なリスト（数字）× 親近感</t>
+          <t>トピック＋ひねり（通説否定）× 比較</t>
         </is>
       </c>
       <c r="I45" s="86" t="inlineStr">
         <is>
-          <t>「スピーキング8.0の私が、Part 3で答えに詰まった時に言うこと3選」</t>
+          <t>「知らない話題に詰まるのは英語力のせいじゃない」／『英語力』に×</t>
         </is>
       </c>
       <c r="J45" s="85" t="n"/>
@@ -4951,51 +4951,19 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="30" customHeight="1" s="35">
+    <row r="46" ht="18" customHeight="1" s="35">
       <c r="A46" s="84">
         <f>IF(C46="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B46" s="85" t="inlineStr">
-        <is>
-          <t>実験</t>
-        </is>
-      </c>
-      <c r="C46" s="86" t="inlineStr">
-        <is>
-          <t>Shorts：リスニング8.5の受講生がやっていた習慣</t>
-        </is>
-      </c>
-      <c r="D46" s="86" t="inlineStr">
-        <is>
-          <t>IELTS Listening（Shorts）</t>
-        </is>
-      </c>
-      <c r="E46" s="85" t="inlineStr">
-        <is>
-          <t>実験枠</t>
-        </is>
-      </c>
-      <c r="F46" s="86" t="inlineStr">
-        <is>
-          <t>Long最大のリスニング（5,057回）をShortsの勝ち型に乗せる。再生上位のShortsにリスニングはまだないので未検証</t>
-        </is>
-      </c>
-      <c r="G46" s="86" t="inlineStr">
-        <is>
-          <t>チュートリアル（Shorts）</t>
-        </is>
-      </c>
-      <c r="H46" s="86" t="inlineStr">
-        <is>
-          <t>親近感 × トピック＋ひねり</t>
-        </is>
-      </c>
-      <c r="I46" s="86" t="inlineStr">
-        <is>
-          <t>「IELTSリスニング8.5を取った受講生がやっていた、たった1つの習慣」</t>
-        </is>
-      </c>
+      <c r="B46" s="85" t="n"/>
+      <c r="C46" s="86" t="n"/>
+      <c r="D46" s="86" t="n"/>
+      <c r="E46" s="85" t="n"/>
+      <c r="F46" s="86" t="n"/>
+      <c r="G46" s="86" t="n"/>
+      <c r="H46" s="86" t="n"/>
+      <c r="I46" s="86" t="n"/>
       <c r="J46" s="85" t="n"/>
       <c r="K46" s="85" t="n"/>
       <c r="L46" s="85" t="n"/>
@@ -5020,51 +4988,19 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="30" customHeight="1" s="35">
+    <row r="47" ht="18" customHeight="1" s="35">
       <c r="A47" s="84">
         <f>IF(C47="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B47" s="85" t="inlineStr">
-        <is>
-          <t>実験</t>
-        </is>
-      </c>
-      <c r="C47" s="86" t="inlineStr">
-        <is>
-          <t>Shorts：ライティング7.0の人が使わない表現3選</t>
-        </is>
-      </c>
-      <c r="D47" s="86" t="inlineStr">
-        <is>
-          <t>IELTS Writing（Shorts）</t>
-        </is>
-      </c>
-      <c r="E47" s="85" t="inlineStr">
-        <is>
-          <t>実験枠</t>
-        </is>
-      </c>
-      <c r="F47" s="86" t="inlineStr">
-        <is>
-          <t>8.0の私型のライティング版。ただしライティングのShorts「IELTSライティングの減点要因を解消する3つの方法」は644回（平均の約0.4倍）で弱い → 要検証</t>
-        </is>
-      </c>
-      <c r="G47" s="86" t="inlineStr">
-        <is>
-          <t>チュートリアル（Shorts）</t>
-        </is>
-      </c>
-      <c r="H47" s="86" t="inlineStr">
-        <is>
-          <t>明確なリスト（数字）× 比較</t>
-        </is>
-      </c>
-      <c r="I47" s="86" t="inlineStr">
-        <is>
-          <t>「IELTSライティング7.0の人が使わない表現3選」</t>
-        </is>
-      </c>
+      <c r="B47" s="85" t="n"/>
+      <c r="C47" s="86" t="n"/>
+      <c r="D47" s="86" t="n"/>
+      <c r="E47" s="85" t="n"/>
+      <c r="F47" s="86" t="n"/>
+      <c r="G47" s="86" t="n"/>
+      <c r="H47" s="86" t="n"/>
+      <c r="I47" s="86" t="n"/>
       <c r="J47" s="85" t="n"/>
       <c r="K47" s="85" t="n"/>
       <c r="L47" s="85" t="n"/>

</xml_diff>